<commit_message>
Versão inicial finalizada, pronta pra uso
</commit_message>
<xml_diff>
--- a/tabela-excel/amostras.xlsx
+++ b/tabela-excel/amostras.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="63">
   <si>
     <t>290426ab</t>
   </si>
@@ -195,661 +195,7 @@
     <t>Amostra</t>
   </si>
   <si>
-    <t>0.0170</t>
-  </si>
-  <si>
-    <t>0.01300</t>
-  </si>
-  <si>
-    <t>0.01200</t>
-  </si>
-  <si>
-    <t>0.00900</t>
-  </si>
-  <si>
-    <t>0.00800</t>
-  </si>
-  <si>
-    <t>0.01000</t>
-  </si>
-  <si>
-    <t>0.01400</t>
-  </si>
-  <si>
-    <t>0.017</t>
-  </si>
-  <si>
-    <t>0.0090</t>
-  </si>
-  <si>
-    <t>0.0080</t>
-  </si>
-  <si>
-    <t>0.0060</t>
-  </si>
-  <si>
-    <t>0.0050</t>
-  </si>
-  <si>
-    <t>0.012</t>
-  </si>
-  <si>
-    <t>0.0100</t>
-  </si>
-  <si>
-    <t>0.0070</t>
-  </si>
-  <si>
-    <t>1300</t>
-  </si>
-  <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>50.5</t>
-  </si>
-  <si>
-    <t>5.23</t>
-  </si>
-  <si>
-    <t>4.83</t>
-  </si>
-  <si>
-    <t>3.12</t>
-  </si>
-  <si>
-    <t>2.03</t>
-  </si>
-  <si>
-    <t>3.31</t>
-  </si>
-  <si>
-    <t>5.63</t>
-  </si>
-  <si>
-    <t>3.88</t>
-  </si>
-  <si>
-    <t>5.71</t>
-  </si>
-  <si>
-    <t>5.04</t>
-  </si>
-  <si>
-    <t>3.64</t>
-  </si>
-  <si>
-    <t>6600</t>
-  </si>
-  <si>
-    <t>4760</t>
-  </si>
-  <si>
-    <t>7597</t>
-  </si>
-  <si>
-    <t>3535</t>
-  </si>
-  <si>
-    <t>3305</t>
-  </si>
-  <si>
-    <t>4768</t>
-  </si>
-  <si>
-    <t>8733</t>
-  </si>
-  <si>
-    <t>7525</t>
-  </si>
-  <si>
-    <t>10334</t>
-  </si>
-  <si>
-    <t>10570</t>
-  </si>
-  <si>
-    <t>8363</t>
-  </si>
-  <si>
-    <t>0.58</t>
-  </si>
-  <si>
-    <t>0.71</t>
-  </si>
-  <si>
-    <t>0.54</t>
-  </si>
-  <si>
-    <t>0.45</t>
-  </si>
-  <si>
-    <t>0.28</t>
-  </si>
-  <si>
-    <t>0.50</t>
-  </si>
-  <si>
-    <t>0.69</t>
-  </si>
-  <si>
-    <t>1.21</t>
-  </si>
-  <si>
-    <t>0.99</t>
-  </si>
-  <si>
-    <t>0.62</t>
-  </si>
-  <si>
-    <t>0.60</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>3.0</t>
-  </si>
-  <si>
-    <t>2.9</t>
-  </si>
-  <si>
-    <t>2.5</t>
-  </si>
-  <si>
-    <t>1.9</t>
-  </si>
-  <si>
-    <t>5.0</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>9.0</t>
-  </si>
-  <si>
-    <t>2.6</t>
-  </si>
-  <si>
-    <t>368</t>
-  </si>
-  <si>
-    <t>2443</t>
-  </si>
-  <si>
-    <t>2190</t>
-  </si>
-  <si>
-    <t>646</t>
-  </si>
-  <si>
-    <t>364</t>
-  </si>
-  <si>
-    <t>1522</t>
-  </si>
-  <si>
-    <t>2214</t>
-  </si>
-  <si>
-    <t>4323</t>
-  </si>
-  <si>
-    <t>4519</t>
-  </si>
-  <si>
-    <t>1608</t>
-  </si>
-  <si>
-    <t>1344</t>
-  </si>
-  <si>
-    <t>26.8</t>
-  </si>
-  <si>
-    <t>15.62</t>
-  </si>
-  <si>
-    <t>17.3</t>
-  </si>
-  <si>
-    <t>10.75</t>
-  </si>
-  <si>
-    <t>10.51</t>
-  </si>
-  <si>
-    <t>14.83</t>
-  </si>
-  <si>
-    <t>18.6</t>
-  </si>
-  <si>
-    <t>19.0</t>
-  </si>
-  <si>
-    <t>24.8</t>
-  </si>
-  <si>
-    <t>24.1</t>
-  </si>
-  <si>
-    <t>21.9</t>
-  </si>
-  <si>
-    <t>246</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>115</t>
-  </si>
-  <si>
-    <t>66</t>
-  </si>
-  <si>
-    <t>67</t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>275</t>
-  </si>
-  <si>
-    <t>179</t>
-  </si>
-  <si>
-    <t>237</t>
-  </si>
-  <si>
-    <t>172</t>
-  </si>
-  <si>
-    <t>131</t>
-  </si>
-  <si>
-    <t>1.6</t>
-  </si>
-  <si>
-    <t>1.16</t>
-  </si>
-  <si>
-    <t>1.13</t>
-  </si>
-  <si>
-    <t>0.79</t>
-  </si>
-  <si>
-    <t>0.90</t>
-  </si>
-  <si>
-    <t>1.25</t>
-  </si>
-  <si>
-    <t>1.8</t>
-  </si>
-  <si>
-    <t>1.5</t>
-  </si>
-  <si>
-    <t>1.3</t>
-  </si>
-  <si>
-    <t>2161</t>
-  </si>
-  <si>
-    <t>1219</t>
-  </si>
-  <si>
-    <t>1877</t>
-  </si>
-  <si>
-    <t>1179</t>
-  </si>
-  <si>
-    <t>1063</t>
-  </si>
-  <si>
-    <t>1491</t>
-  </si>
-  <si>
-    <t>2071</t>
-  </si>
-  <si>
-    <t>2080</t>
-  </si>
-  <si>
-    <t>2417</t>
-  </si>
-  <si>
-    <t>2385</t>
-  </si>
-  <si>
-    <t>1831</t>
-  </si>
-  <si>
-    <t>9600</t>
-  </si>
-  <si>
-    <t>3362</t>
-  </si>
-  <si>
-    <t>2268</t>
-  </si>
-  <si>
-    <t>2015</t>
-  </si>
-  <si>
-    <t>1987</t>
-  </si>
-  <si>
-    <t>2262</t>
-  </si>
-  <si>
-    <t>2764</t>
-  </si>
-  <si>
-    <t>2530</t>
-  </si>
-  <si>
-    <t>2707</t>
-  </si>
-  <si>
-    <t>2773</t>
-  </si>
-  <si>
-    <t>2272</t>
-  </si>
-  <si>
-    <t>0.054</t>
-  </si>
-  <si>
-    <t>85</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>0.0003</t>
-  </si>
-  <si>
-    <t>0.00025</t>
-  </si>
-  <si>
-    <t>0.00023</t>
-  </si>
-  <si>
-    <t>0.00018</t>
-  </si>
-  <si>
-    <t>0.00016</t>
-  </si>
-  <si>
-    <t>0.00019</t>
-  </si>
-  <si>
-    <t>0.00027</t>
-  </si>
-  <si>
-    <t>0.004</t>
-  </si>
-  <si>
-    <t>0.0025</t>
-  </si>
-  <si>
-    <t>0.0022</t>
-  </si>
-  <si>
-    <t>0.0020</t>
-  </si>
-  <si>
-    <t>0.0018</t>
-  </si>
-  <si>
-    <t>0.003</t>
-  </si>
-  <si>
-    <t>0.0029</t>
-  </si>
-  <si>
-    <t>0.0027</t>
-  </si>
-  <si>
-    <t>0.0023</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>0.6</t>
-  </si>
-  <si>
-    <t>0.07</t>
-  </si>
-  <si>
-    <t>0.05</t>
-  </si>
-  <si>
-    <t>0.04</t>
-  </si>
-  <si>
-    <t>0.08</t>
-  </si>
-  <si>
-    <t>0.06</t>
-  </si>
-  <si>
-    <t>82</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>83</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>57</t>
-  </si>
-  <si>
-    <t>94</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>112</t>
-  </si>
-  <si>
-    <t>91</t>
-  </si>
-  <si>
-    <t>0.10</t>
-  </si>
-  <si>
-    <t>0.11</t>
-  </si>
-  <si>
-    <t>0.09</t>
-  </si>
-  <si>
-    <t>0.16</t>
-  </si>
-  <si>
-    <t>0.14</t>
-  </si>
-  <si>
-    <t>0.8</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>0.9</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t>93</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>0.30</t>
-  </si>
-  <si>
-    <t>0.3</t>
-  </si>
-  <si>
-    <t>0.21</t>
-  </si>
-  <si>
-    <t>0.20</t>
-  </si>
-  <si>
-    <t>0.4</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>0.29</t>
-  </si>
-  <si>
-    <t>0.26</t>
-  </si>
-  <si>
-    <t>0.18</t>
-  </si>
-  <si>
-    <t>0.23</t>
-  </si>
-  <si>
-    <t>320</t>
-  </si>
-  <si>
-    <t>194</t>
-  </si>
-  <si>
-    <t>245</t>
-  </si>
-  <si>
-    <t>171</t>
-  </si>
-  <si>
-    <t>150</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>274</t>
-  </si>
-  <si>
-    <t>271</t>
-  </si>
-  <si>
-    <t>316</t>
-  </si>
-  <si>
-    <t>309</t>
-  </si>
-  <si>
-    <t>248</t>
-  </si>
-  <si>
-    <t>181</t>
-  </si>
-  <si>
-    <t>87</t>
-  </si>
-  <si>
-    <t>71</t>
-  </si>
-  <si>
-    <t>61</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>84</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>88</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>0.026</t>
-  </si>
-  <si>
-    <t>15</t>
   </si>
   <si>
     <t>LD</t>
@@ -6818,616 +6164,616 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" t="s">
-        <v>98</v>
-      </c>
-      <c r="H2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I2" t="s">
-        <v>114</v>
-      </c>
-      <c r="J2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K2" t="s">
-        <v>129</v>
-      </c>
-      <c r="L2" t="s">
-        <v>140</v>
-      </c>
-      <c r="M2" t="s">
-        <v>151</v>
-      </c>
-      <c r="N2" t="s">
-        <v>160</v>
-      </c>
-      <c r="O2" t="s">
-        <v>171</v>
-      </c>
-      <c r="P2" t="s">
-        <v>182</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>183</v>
-      </c>
-      <c r="R2" t="s">
-        <v>184</v>
+      <c r="B2">
+        <v>0.017</v>
+      </c>
+      <c r="C2">
+        <v>0.017</v>
+      </c>
+      <c r="D2">
+        <v>1300</v>
+      </c>
+      <c r="E2">
+        <v>50.5</v>
+      </c>
+      <c r="F2">
+        <v>6600</v>
+      </c>
+      <c r="G2">
+        <v>0.58</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2">
+        <v>368</v>
+      </c>
+      <c r="K2">
+        <v>26.8</v>
+      </c>
+      <c r="L2">
+        <v>246</v>
+      </c>
+      <c r="M2">
+        <v>1.6</v>
+      </c>
+      <c r="N2">
+        <v>2161</v>
+      </c>
+      <c r="O2">
+        <v>9600</v>
+      </c>
+      <c r="P2">
+        <v>0.054</v>
+      </c>
+      <c r="Q2">
+        <v>85</v>
+      </c>
+      <c r="R2">
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" t="s">
-        <v>67</v>
+      <c r="B3">
+        <v>0.013</v>
+      </c>
+      <c r="C3">
+        <v>0.008999999999999999</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G3" t="s">
-        <v>99</v>
-      </c>
-      <c r="H3" t="s">
-        <v>110</v>
+        <v>59</v>
+      </c>
+      <c r="E3">
+        <v>5.23</v>
+      </c>
+      <c r="F3">
+        <v>4760</v>
+      </c>
+      <c r="G3">
+        <v>0.71</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
-      </c>
-      <c r="J3" t="s">
-        <v>119</v>
-      </c>
-      <c r="K3" t="s">
-        <v>130</v>
-      </c>
-      <c r="L3" t="s">
-        <v>141</v>
-      </c>
-      <c r="M3" t="s">
-        <v>152</v>
-      </c>
-      <c r="N3" t="s">
-        <v>161</v>
-      </c>
-      <c r="O3" t="s">
-        <v>172</v>
+        <v>59</v>
+      </c>
+      <c r="J3">
+        <v>2443</v>
+      </c>
+      <c r="K3">
+        <v>15.62</v>
+      </c>
+      <c r="L3">
+        <v>101</v>
+      </c>
+      <c r="M3">
+        <v>1.16</v>
+      </c>
+      <c r="N3">
+        <v>1219</v>
+      </c>
+      <c r="O3">
+        <v>3362</v>
       </c>
       <c r="P3" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q3" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="R3" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:18">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" t="s">
-        <v>68</v>
+      <c r="B4">
+        <v>0.012</v>
+      </c>
+      <c r="C4">
+        <v>0.008</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" t="s">
-        <v>100</v>
-      </c>
-      <c r="H4" t="s">
-        <v>111</v>
+        <v>59</v>
+      </c>
+      <c r="E4">
+        <v>4.83</v>
+      </c>
+      <c r="F4">
+        <v>7597</v>
+      </c>
+      <c r="G4">
+        <v>0.54</v>
+      </c>
+      <c r="H4">
+        <v>2.9</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
-      </c>
-      <c r="J4" t="s">
-        <v>120</v>
-      </c>
-      <c r="K4" t="s">
-        <v>131</v>
-      </c>
-      <c r="L4" t="s">
-        <v>142</v>
-      </c>
-      <c r="M4" t="s">
-        <v>153</v>
-      </c>
-      <c r="N4" t="s">
-        <v>162</v>
-      </c>
-      <c r="O4" t="s">
-        <v>173</v>
+        <v>59</v>
+      </c>
+      <c r="J4">
+        <v>2190</v>
+      </c>
+      <c r="K4">
+        <v>17.3</v>
+      </c>
+      <c r="L4">
+        <v>115</v>
+      </c>
+      <c r="M4">
+        <v>1.13</v>
+      </c>
+      <c r="N4">
+        <v>1877</v>
+      </c>
+      <c r="O4">
+        <v>2268</v>
       </c>
       <c r="P4" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q4" t="s">
-        <v>75</v>
-      </c>
-      <c r="R4" t="s">
-        <v>115</v>
+        <v>59</v>
+      </c>
+      <c r="R4">
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" t="s">
-        <v>69</v>
+      <c r="B5">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="C5">
+        <v>0.006</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" t="s">
-        <v>101</v>
-      </c>
-      <c r="H5" t="s">
-        <v>112</v>
+        <v>59</v>
+      </c>
+      <c r="E5">
+        <v>3.12</v>
+      </c>
+      <c r="F5">
+        <v>3535</v>
+      </c>
+      <c r="G5">
+        <v>0.45</v>
+      </c>
+      <c r="H5">
+        <v>2.5</v>
       </c>
       <c r="I5" t="s">
-        <v>75</v>
-      </c>
-      <c r="J5" t="s">
-        <v>121</v>
-      </c>
-      <c r="K5" t="s">
-        <v>132</v>
-      </c>
-      <c r="L5" t="s">
-        <v>143</v>
-      </c>
-      <c r="M5" t="s">
-        <v>154</v>
-      </c>
-      <c r="N5" t="s">
-        <v>163</v>
-      </c>
-      <c r="O5" t="s">
-        <v>174</v>
+        <v>59</v>
+      </c>
+      <c r="J5">
+        <v>646</v>
+      </c>
+      <c r="K5">
+        <v>10.75</v>
+      </c>
+      <c r="L5">
+        <v>66</v>
+      </c>
+      <c r="M5">
+        <v>0.79</v>
+      </c>
+      <c r="N5">
+        <v>1179</v>
+      </c>
+      <c r="O5">
+        <v>2015</v>
       </c>
       <c r="P5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q5" t="s">
-        <v>75</v>
-      </c>
-      <c r="R5" t="s">
-        <v>185</v>
+        <v>59</v>
+      </c>
+      <c r="R5">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:18">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" t="s">
-        <v>70</v>
+      <c r="B6">
+        <v>0.008</v>
+      </c>
+      <c r="C6">
+        <v>0.005</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G6" t="s">
-        <v>102</v>
-      </c>
-      <c r="H6" t="s">
-        <v>113</v>
+        <v>59</v>
+      </c>
+      <c r="E6">
+        <v>2.03</v>
+      </c>
+      <c r="F6">
+        <v>3305</v>
+      </c>
+      <c r="G6">
+        <v>0.28</v>
+      </c>
+      <c r="H6">
+        <v>1.9</v>
       </c>
       <c r="I6" t="s">
-        <v>75</v>
-      </c>
-      <c r="J6" t="s">
-        <v>122</v>
-      </c>
-      <c r="K6" t="s">
-        <v>133</v>
-      </c>
-      <c r="L6" t="s">
-        <v>144</v>
-      </c>
-      <c r="M6" t="s">
-        <v>104</v>
-      </c>
-      <c r="N6" t="s">
-        <v>164</v>
-      </c>
-      <c r="O6" t="s">
-        <v>175</v>
+        <v>59</v>
+      </c>
+      <c r="J6">
+        <v>364</v>
+      </c>
+      <c r="K6">
+        <v>10.51</v>
+      </c>
+      <c r="L6">
+        <v>67</v>
+      </c>
+      <c r="M6">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="N6">
+        <v>1063</v>
+      </c>
+      <c r="O6">
+        <v>1987</v>
       </c>
       <c r="P6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="R6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" t="s">
-        <v>70</v>
+      <c r="B7">
+        <v>0.01</v>
+      </c>
+      <c r="C7">
+        <v>0.005</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" t="s">
-        <v>103</v>
-      </c>
-      <c r="H7" t="s">
-        <v>111</v>
+        <v>59</v>
+      </c>
+      <c r="E7">
+        <v>3.31</v>
+      </c>
+      <c r="F7">
+        <v>4768</v>
+      </c>
+      <c r="G7">
+        <v>0.5</v>
+      </c>
+      <c r="H7">
+        <v>2.9</v>
       </c>
       <c r="I7" t="s">
-        <v>75</v>
-      </c>
-      <c r="J7" t="s">
-        <v>123</v>
-      </c>
-      <c r="K7" t="s">
-        <v>134</v>
-      </c>
-      <c r="L7" t="s">
-        <v>145</v>
-      </c>
-      <c r="M7" t="s">
-        <v>155</v>
-      </c>
-      <c r="N7" t="s">
-        <v>165</v>
-      </c>
-      <c r="O7" t="s">
-        <v>176</v>
+        <v>59</v>
+      </c>
+      <c r="J7">
+        <v>1522</v>
+      </c>
+      <c r="K7">
+        <v>14.83</v>
+      </c>
+      <c r="L7">
+        <v>95</v>
+      </c>
+      <c r="M7">
+        <v>0.9</v>
+      </c>
+      <c r="N7">
+        <v>1491</v>
+      </c>
+      <c r="O7">
+        <v>2262</v>
       </c>
       <c r="P7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
-        <v>75</v>
-      </c>
-      <c r="R7" t="s">
-        <v>115</v>
+        <v>59</v>
+      </c>
+      <c r="R7">
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:18">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" t="s">
-        <v>68</v>
+      <c r="B8">
+        <v>0.013</v>
+      </c>
+      <c r="C8">
+        <v>0.008</v>
       </c>
       <c r="D8" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F8" t="s">
-        <v>93</v>
-      </c>
-      <c r="G8" t="s">
-        <v>104</v>
-      </c>
-      <c r="H8" t="s">
-        <v>114</v>
+        <v>59</v>
+      </c>
+      <c r="E8">
+        <v>5.63</v>
+      </c>
+      <c r="F8">
+        <v>8733</v>
+      </c>
+      <c r="G8">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
       </c>
       <c r="I8" t="s">
-        <v>75</v>
-      </c>
-      <c r="J8" t="s">
-        <v>124</v>
-      </c>
-      <c r="K8" t="s">
-        <v>135</v>
-      </c>
-      <c r="L8" t="s">
-        <v>146</v>
-      </c>
-      <c r="M8" t="s">
-        <v>156</v>
-      </c>
-      <c r="N8" t="s">
-        <v>166</v>
-      </c>
-      <c r="O8" t="s">
-        <v>177</v>
+        <v>59</v>
+      </c>
+      <c r="J8">
+        <v>2214</v>
+      </c>
+      <c r="K8">
+        <v>18.6</v>
+      </c>
+      <c r="L8">
+        <v>275</v>
+      </c>
+      <c r="M8">
+        <v>1.25</v>
+      </c>
+      <c r="N8">
+        <v>2071</v>
+      </c>
+      <c r="O8">
+        <v>2764</v>
       </c>
       <c r="P8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q8" t="s">
-        <v>75</v>
-      </c>
-      <c r="R8" t="s">
-        <v>186</v>
+        <v>59</v>
+      </c>
+      <c r="R8">
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:18">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" t="s">
-        <v>71</v>
+      <c r="B9">
+        <v>0.012</v>
+      </c>
+      <c r="C9">
+        <v>0.012</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9" t="s">
-        <v>115</v>
+        <v>59</v>
+      </c>
+      <c r="E9">
+        <v>3.88</v>
+      </c>
+      <c r="F9">
+        <v>7525</v>
+      </c>
+      <c r="G9">
+        <v>1.21</v>
+      </c>
+      <c r="H9">
+        <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
-      </c>
-      <c r="J9" t="s">
-        <v>125</v>
-      </c>
-      <c r="K9" t="s">
-        <v>136</v>
-      </c>
-      <c r="L9" t="s">
-        <v>147</v>
-      </c>
-      <c r="M9" t="s">
-        <v>157</v>
-      </c>
-      <c r="N9" t="s">
-        <v>167</v>
-      </c>
-      <c r="O9" t="s">
-        <v>178</v>
+        <v>59</v>
+      </c>
+      <c r="J9">
+        <v>4323</v>
+      </c>
+      <c r="K9">
+        <v>19</v>
+      </c>
+      <c r="L9">
+        <v>179</v>
+      </c>
+      <c r="M9">
+        <v>1.8</v>
+      </c>
+      <c r="N9">
+        <v>2080</v>
+      </c>
+      <c r="O9">
+        <v>2530</v>
       </c>
       <c r="P9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q9" t="s">
-        <v>75</v>
-      </c>
-      <c r="R9" t="s">
-        <v>187</v>
+        <v>59</v>
+      </c>
+      <c r="R9">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:18">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" t="s">
-        <v>67</v>
+      <c r="B10">
+        <v>0.014</v>
+      </c>
+      <c r="C10">
+        <v>0.008999999999999999</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
-      </c>
-      <c r="E10" t="s">
-        <v>84</v>
-      </c>
-      <c r="F10" t="s">
-        <v>95</v>
-      </c>
-      <c r="G10" t="s">
-        <v>106</v>
-      </c>
-      <c r="H10" t="s">
-        <v>116</v>
+        <v>59</v>
+      </c>
+      <c r="E10">
+        <v>5.71</v>
+      </c>
+      <c r="F10">
+        <v>10334</v>
+      </c>
+      <c r="G10">
+        <v>0.99</v>
+      </c>
+      <c r="H10">
+        <v>9</v>
       </c>
       <c r="I10" t="s">
-        <v>75</v>
-      </c>
-      <c r="J10" t="s">
-        <v>126</v>
-      </c>
-      <c r="K10" t="s">
-        <v>137</v>
-      </c>
-      <c r="L10" t="s">
-        <v>148</v>
-      </c>
-      <c r="M10" t="s">
-        <v>158</v>
-      </c>
-      <c r="N10" t="s">
-        <v>168</v>
-      </c>
-      <c r="O10" t="s">
-        <v>179</v>
+        <v>59</v>
+      </c>
+      <c r="J10">
+        <v>4519</v>
+      </c>
+      <c r="K10">
+        <v>24.8</v>
+      </c>
+      <c r="L10">
+        <v>237</v>
+      </c>
+      <c r="M10">
+        <v>1.5</v>
+      </c>
+      <c r="N10">
+        <v>2417</v>
+      </c>
+      <c r="O10">
+        <v>2707</v>
       </c>
       <c r="P10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R10" t="s">
-        <v>188</v>
+        <v>59</v>
+      </c>
+      <c r="R10">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:18">
       <c r="A11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" t="s">
-        <v>72</v>
+      <c r="B11">
+        <v>0.014</v>
+      </c>
+      <c r="C11">
+        <v>0.01</v>
       </c>
       <c r="D11" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" t="s">
-        <v>96</v>
-      </c>
-      <c r="G11" t="s">
-        <v>107</v>
-      </c>
-      <c r="H11" t="s">
-        <v>110</v>
+        <v>59</v>
+      </c>
+      <c r="E11">
+        <v>5.04</v>
+      </c>
+      <c r="F11">
+        <v>10570</v>
+      </c>
+      <c r="G11">
+        <v>0.62</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J11" t="s">
-        <v>127</v>
-      </c>
-      <c r="K11" t="s">
-        <v>138</v>
-      </c>
-      <c r="L11" t="s">
-        <v>149</v>
-      </c>
-      <c r="M11" t="s">
-        <v>159</v>
-      </c>
-      <c r="N11" t="s">
-        <v>169</v>
-      </c>
-      <c r="O11" t="s">
-        <v>180</v>
+        <v>59</v>
+      </c>
+      <c r="J11">
+        <v>1608</v>
+      </c>
+      <c r="K11">
+        <v>24.1</v>
+      </c>
+      <c r="L11">
+        <v>172</v>
+      </c>
+      <c r="M11">
+        <v>1.3</v>
+      </c>
+      <c r="N11">
+        <v>2385</v>
+      </c>
+      <c r="O11">
+        <v>2773</v>
       </c>
       <c r="P11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q11" t="s">
-        <v>75</v>
-      </c>
-      <c r="R11" t="s">
-        <v>189</v>
+        <v>59</v>
+      </c>
+      <c r="R11">
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" t="s">
-        <v>73</v>
+      <c r="B12">
+        <v>0.013</v>
+      </c>
+      <c r="C12">
+        <v>0.007</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" t="s">
-        <v>86</v>
-      </c>
-      <c r="F12" t="s">
-        <v>97</v>
-      </c>
-      <c r="G12" t="s">
-        <v>108</v>
-      </c>
-      <c r="H12" t="s">
-        <v>117</v>
+        <v>59</v>
+      </c>
+      <c r="E12">
+        <v>3.64</v>
+      </c>
+      <c r="F12">
+        <v>8363</v>
+      </c>
+      <c r="G12">
+        <v>0.6</v>
+      </c>
+      <c r="H12">
+        <v>2.6</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
-      </c>
-      <c r="J12" t="s">
-        <v>128</v>
-      </c>
-      <c r="K12" t="s">
-        <v>139</v>
-      </c>
-      <c r="L12" t="s">
-        <v>150</v>
-      </c>
-      <c r="M12" t="s">
-        <v>158</v>
-      </c>
-      <c r="N12" t="s">
-        <v>170</v>
-      </c>
-      <c r="O12" t="s">
-        <v>181</v>
+        <v>59</v>
+      </c>
+      <c r="J12">
+        <v>1344</v>
+      </c>
+      <c r="K12">
+        <v>21.9</v>
+      </c>
+      <c r="L12">
+        <v>131</v>
+      </c>
+      <c r="M12">
+        <v>1.5</v>
+      </c>
+      <c r="N12">
+        <v>1831</v>
+      </c>
+      <c r="O12">
+        <v>2272</v>
       </c>
       <c r="P12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q12" t="s">
-        <v>75</v>
-      </c>
-      <c r="R12" t="s">
-        <v>190</v>
+        <v>59</v>
+      </c>
+      <c r="R12">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -7495,1339 +6841,1339 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" t="s">
-        <v>278</v>
-      </c>
-      <c r="B2">
-        <v>0.00027</v>
-      </c>
-      <c r="D2">
-        <v>0.006</v>
-      </c>
-      <c r="F2">
-        <v>13</v>
-      </c>
-      <c r="H2">
-        <v>0.05</v>
-      </c>
-      <c r="J2">
-        <v>70</v>
-      </c>
-      <c r="L2">
-        <v>0.14</v>
-      </c>
-      <c r="N2">
-        <v>1.2</v>
-      </c>
-      <c r="P2">
-        <v>1.6</v>
-      </c>
-      <c r="R2">
-        <v>9</v>
-      </c>
-      <c r="T2">
-        <v>0.08</v>
-      </c>
-      <c r="V2">
-        <v>13</v>
-      </c>
-      <c r="X2">
-        <v>0.3</v>
-      </c>
-      <c r="Z2">
-        <v>400</v>
-      </c>
-      <c r="AB2">
-        <v>170</v>
-      </c>
-      <c r="AD2">
-        <v>0.025</v>
-      </c>
-      <c r="AF2">
-        <v>14</v>
-      </c>
-      <c r="AH2">
-        <v>8</v>
+        <v>60</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J2" t="s">
+        <v>59</v>
+      </c>
+      <c r="L2" t="s">
+        <v>59</v>
+      </c>
+      <c r="N2" t="s">
+        <v>59</v>
+      </c>
+      <c r="P2" t="s">
+        <v>59</v>
+      </c>
+      <c r="R2" t="s">
+        <v>59</v>
+      </c>
+      <c r="T2" t="s">
+        <v>59</v>
+      </c>
+      <c r="V2" t="s">
+        <v>59</v>
+      </c>
+      <c r="X2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:35">
       <c r="B3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="G3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="J3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="K3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="L3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="M3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="N3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="O3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="P3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="Q3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="R3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="S3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="T3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="U3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="V3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="W3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="X3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="Y3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="Z3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="AA3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="AB3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="AC3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="AD3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="AE3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="AF3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="AG3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="AH3" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="AI3" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" t="s">
-        <v>74</v>
-      </c>
-      <c r="G4" t="s">
-        <v>207</v>
-      </c>
-      <c r="H4" t="s">
-        <v>76</v>
-      </c>
-      <c r="I4" t="s">
-        <v>208</v>
-      </c>
-      <c r="J4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K4" t="s">
-        <v>214</v>
-      </c>
-      <c r="L4" t="s">
-        <v>98</v>
-      </c>
-      <c r="M4" t="s">
-        <v>224</v>
-      </c>
-      <c r="N4" t="s">
-        <v>109</v>
-      </c>
-      <c r="O4" t="s">
-        <v>229</v>
-      </c>
-      <c r="P4" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>109</v>
-      </c>
-      <c r="R4" t="s">
-        <v>118</v>
-      </c>
-      <c r="S4" t="s">
-        <v>185</v>
-      </c>
-      <c r="T4" t="s">
-        <v>129</v>
-      </c>
-      <c r="U4" t="s">
-        <v>240</v>
-      </c>
-      <c r="V4" t="s">
-        <v>140</v>
-      </c>
-      <c r="W4" t="s">
+      <c r="B4">
+        <v>0.017</v>
+      </c>
+      <c r="C4">
+        <v>0.0003</v>
+      </c>
+      <c r="D4">
+        <v>0.017</v>
+      </c>
+      <c r="E4">
+        <v>0.004</v>
+      </c>
+      <c r="F4">
+        <v>1300</v>
+      </c>
+      <c r="G4">
+        <v>19</v>
+      </c>
+      <c r="H4">
+        <v>50.5</v>
+      </c>
+      <c r="I4">
+        <v>0.6</v>
+      </c>
+      <c r="J4">
+        <v>6600</v>
+      </c>
+      <c r="K4">
+        <v>82</v>
+      </c>
+      <c r="L4">
+        <v>0.58</v>
+      </c>
+      <c r="M4">
+        <v>0.1</v>
+      </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
+      <c r="O4">
+        <v>0.8</v>
+      </c>
+      <c r="P4">
+        <v>5</v>
+      </c>
+      <c r="Q4">
+        <v>2</v>
+      </c>
+      <c r="R4">
+        <v>368</v>
+      </c>
+      <c r="S4">
+        <v>10</v>
+      </c>
+      <c r="T4">
+        <v>26.8</v>
+      </c>
+      <c r="U4">
+        <v>0.5</v>
+      </c>
+      <c r="V4">
         <v>246</v>
       </c>
-      <c r="X4" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>160</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>256</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>171</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>267</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>182</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>276</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>183</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>277</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>184</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>247</v>
+      <c r="W4">
+        <v>13</v>
+      </c>
+      <c r="X4">
+        <v>1.6</v>
+      </c>
+      <c r="Y4">
+        <v>0.3</v>
+      </c>
+      <c r="Z4">
+        <v>2161</v>
+      </c>
+      <c r="AA4">
+        <v>320</v>
+      </c>
+      <c r="AB4">
+        <v>9600</v>
+      </c>
+      <c r="AC4">
+        <v>181</v>
+      </c>
+      <c r="AD4">
+        <v>0.054</v>
+      </c>
+      <c r="AE4">
+        <v>0.026</v>
+      </c>
+      <c r="AF4">
+        <v>85</v>
+      </c>
+      <c r="AG4">
+        <v>15</v>
+      </c>
+      <c r="AH4">
+        <v>31</v>
+      </c>
+      <c r="AI4">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:35">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" t="s">
-        <v>192</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>199</v>
+      <c r="B5">
+        <v>0.013</v>
+      </c>
+      <c r="C5">
+        <v>0.00025</v>
+      </c>
+      <c r="D5">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E5">
+        <v>0.0025</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
-      </c>
-      <c r="H5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" t="s">
-        <v>209</v>
-      </c>
-      <c r="J5" t="s">
-        <v>88</v>
-      </c>
-      <c r="K5" t="s">
-        <v>215</v>
-      </c>
-      <c r="L5" t="s">
-        <v>99</v>
-      </c>
-      <c r="M5" t="s">
-        <v>225</v>
-      </c>
-      <c r="N5" t="s">
-        <v>110</v>
-      </c>
-      <c r="O5" t="s">
-        <v>230</v>
+        <v>59</v>
+      </c>
+      <c r="H5">
+        <v>5.23</v>
+      </c>
+      <c r="I5">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J5">
+        <v>4760</v>
+      </c>
+      <c r="K5">
+        <v>59</v>
+      </c>
+      <c r="L5">
+        <v>0.71</v>
+      </c>
+      <c r="M5">
+        <v>0.11</v>
+      </c>
+      <c r="N5">
+        <v>3</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
       </c>
       <c r="P5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q5" t="s">
-        <v>75</v>
-      </c>
-      <c r="R5" t="s">
-        <v>119</v>
-      </c>
-      <c r="S5" t="s">
-        <v>233</v>
-      </c>
-      <c r="T5" t="s">
-        <v>130</v>
-      </c>
-      <c r="U5" t="s">
-        <v>241</v>
-      </c>
-      <c r="V5" t="s">
-        <v>141</v>
-      </c>
-      <c r="W5" t="s">
-        <v>247</v>
-      </c>
-      <c r="X5" t="s">
-        <v>152</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>252</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>161</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>257</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>268</v>
+        <v>59</v>
+      </c>
+      <c r="R5">
+        <v>2443</v>
+      </c>
+      <c r="S5">
+        <v>51</v>
+      </c>
+      <c r="T5">
+        <v>15.62</v>
+      </c>
+      <c r="U5">
+        <v>0.3</v>
+      </c>
+      <c r="V5">
+        <v>101</v>
+      </c>
+      <c r="W5">
+        <v>8</v>
+      </c>
+      <c r="X5">
+        <v>1.16</v>
+      </c>
+      <c r="Y5">
+        <v>0.29</v>
+      </c>
+      <c r="Z5">
+        <v>1219</v>
+      </c>
+      <c r="AA5">
+        <v>194</v>
+      </c>
+      <c r="AB5">
+        <v>3362</v>
+      </c>
+      <c r="AC5">
+        <v>87</v>
       </c>
       <c r="AD5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AH5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AI5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:35">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" t="s">
-        <v>200</v>
+      <c r="B6">
+        <v>0.012</v>
+      </c>
+      <c r="C6">
+        <v>0.00023</v>
+      </c>
+      <c r="D6">
+        <v>0.008</v>
+      </c>
+      <c r="E6">
+        <v>0.0022</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" t="s">
-        <v>78</v>
-      </c>
-      <c r="I6" t="s">
-        <v>209</v>
-      </c>
-      <c r="J6" t="s">
-        <v>89</v>
-      </c>
-      <c r="K6" t="s">
-        <v>216</v>
-      </c>
-      <c r="L6" t="s">
-        <v>100</v>
-      </c>
-      <c r="M6" t="s">
-        <v>226</v>
-      </c>
-      <c r="N6" t="s">
-        <v>111</v>
-      </c>
-      <c r="O6" t="s">
-        <v>231</v>
+        <v>59</v>
+      </c>
+      <c r="H6">
+        <v>4.83</v>
+      </c>
+      <c r="I6">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J6">
+        <v>7597</v>
+      </c>
+      <c r="K6">
+        <v>83</v>
+      </c>
+      <c r="L6">
+        <v>0.54</v>
+      </c>
+      <c r="M6">
+        <v>0.09</v>
+      </c>
+      <c r="N6">
+        <v>2.9</v>
+      </c>
+      <c r="O6">
+        <v>0.9</v>
       </c>
       <c r="P6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q6" t="s">
-        <v>75</v>
-      </c>
-      <c r="R6" t="s">
-        <v>120</v>
-      </c>
-      <c r="S6" t="s">
-        <v>217</v>
-      </c>
-      <c r="T6" t="s">
-        <v>131</v>
-      </c>
-      <c r="U6" t="s">
-        <v>242</v>
-      </c>
-      <c r="V6" t="s">
-        <v>142</v>
-      </c>
-      <c r="W6" t="s">
-        <v>247</v>
-      </c>
-      <c r="X6" t="s">
-        <v>153</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>253</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>258</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>173</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>269</v>
+        <v>59</v>
+      </c>
+      <c r="R6">
+        <v>2190</v>
+      </c>
+      <c r="S6">
+        <v>46</v>
+      </c>
+      <c r="T6">
+        <v>17.3</v>
+      </c>
+      <c r="U6">
+        <v>0.3</v>
+      </c>
+      <c r="V6">
+        <v>115</v>
+      </c>
+      <c r="W6">
+        <v>8</v>
+      </c>
+      <c r="X6">
+        <v>1.13</v>
+      </c>
+      <c r="Y6">
+        <v>0.26</v>
+      </c>
+      <c r="Z6">
+        <v>1877</v>
+      </c>
+      <c r="AA6">
+        <v>245</v>
+      </c>
+      <c r="AB6">
+        <v>2268</v>
+      </c>
+      <c r="AC6">
+        <v>71</v>
       </c>
       <c r="AD6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF6" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>115</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>249</v>
+        <v>59</v>
+      </c>
+      <c r="AH6">
+        <v>16</v>
+      </c>
+      <c r="AI6">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:35">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" t="s">
-        <v>194</v>
-      </c>
-      <c r="D7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" t="s">
-        <v>201</v>
+      <c r="B7">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0.00018</v>
+      </c>
+      <c r="D7">
+        <v>0.006</v>
+      </c>
+      <c r="E7">
+        <v>0.002</v>
       </c>
       <c r="F7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G7" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" t="s">
-        <v>79</v>
-      </c>
-      <c r="I7" t="s">
-        <v>210</v>
-      </c>
-      <c r="J7" t="s">
-        <v>90</v>
-      </c>
-      <c r="K7" t="s">
-        <v>217</v>
-      </c>
-      <c r="L7" t="s">
-        <v>101</v>
-      </c>
-      <c r="M7" t="s">
-        <v>209</v>
-      </c>
-      <c r="N7" t="s">
-        <v>112</v>
-      </c>
-      <c r="O7" t="s">
-        <v>229</v>
+        <v>59</v>
+      </c>
+      <c r="H7">
+        <v>3.12</v>
+      </c>
+      <c r="I7">
+        <v>0.05</v>
+      </c>
+      <c r="J7">
+        <v>3535</v>
+      </c>
+      <c r="K7">
+        <v>46</v>
+      </c>
+      <c r="L7">
+        <v>0.45</v>
+      </c>
+      <c r="M7">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="N7">
+        <v>2.5</v>
+      </c>
+      <c r="O7">
+        <v>0.8</v>
       </c>
       <c r="P7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
-        <v>75</v>
-      </c>
-      <c r="R7" t="s">
-        <v>121</v>
-      </c>
-      <c r="S7" t="s">
-        <v>234</v>
-      </c>
-      <c r="T7" t="s">
-        <v>132</v>
-      </c>
-      <c r="U7" t="s">
-        <v>243</v>
-      </c>
-      <c r="V7" t="s">
-        <v>143</v>
-      </c>
-      <c r="W7" t="s">
-        <v>248</v>
-      </c>
-      <c r="X7" t="s">
-        <v>154</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>243</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>259</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>174</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>270</v>
+        <v>59</v>
+      </c>
+      <c r="R7">
+        <v>646</v>
+      </c>
+      <c r="S7">
+        <v>14</v>
+      </c>
+      <c r="T7">
+        <v>10.75</v>
+      </c>
+      <c r="U7">
+        <v>0.21</v>
+      </c>
+      <c r="V7">
+        <v>66</v>
+      </c>
+      <c r="W7">
+        <v>6</v>
+      </c>
+      <c r="X7">
+        <v>0.79</v>
+      </c>
+      <c r="Y7">
+        <v>0.21</v>
+      </c>
+      <c r="Z7">
+        <v>1179</v>
+      </c>
+      <c r="AA7">
+        <v>171</v>
+      </c>
+      <c r="AB7">
+        <v>2015</v>
+      </c>
+      <c r="AC7">
+        <v>61</v>
       </c>
       <c r="AD7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF7" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG7" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>185</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>232</v>
+        <v>59</v>
+      </c>
+      <c r="AH7">
+        <v>10</v>
+      </c>
+      <c r="AI7">
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:35">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" t="s">
-        <v>195</v>
-      </c>
-      <c r="D8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" t="s">
-        <v>202</v>
+      <c r="B8">
+        <v>0.008</v>
+      </c>
+      <c r="C8">
+        <v>0.00016</v>
+      </c>
+      <c r="D8">
+        <v>0.005</v>
+      </c>
+      <c r="E8">
+        <v>0.0018</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G8" t="s">
-        <v>75</v>
-      </c>
-      <c r="H8" t="s">
-        <v>80</v>
-      </c>
-      <c r="I8" t="s">
-        <v>211</v>
-      </c>
-      <c r="J8" t="s">
-        <v>91</v>
-      </c>
-      <c r="K8" t="s">
-        <v>218</v>
-      </c>
-      <c r="L8" t="s">
-        <v>102</v>
-      </c>
-      <c r="M8" t="s">
-        <v>210</v>
-      </c>
-      <c r="N8" t="s">
-        <v>113</v>
-      </c>
-      <c r="O8" t="s">
-        <v>208</v>
+        <v>59</v>
+      </c>
+      <c r="H8">
+        <v>2.03</v>
+      </c>
+      <c r="I8">
+        <v>0.04</v>
+      </c>
+      <c r="J8">
+        <v>3305</v>
+      </c>
+      <c r="K8">
+        <v>42</v>
+      </c>
+      <c r="L8">
+        <v>0.28</v>
+      </c>
+      <c r="M8">
+        <v>0.05</v>
+      </c>
+      <c r="N8">
+        <v>1.9</v>
+      </c>
+      <c r="O8">
+        <v>0.6</v>
       </c>
       <c r="P8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q8" t="s">
-        <v>75</v>
-      </c>
-      <c r="R8" t="s">
-        <v>122</v>
-      </c>
-      <c r="S8" t="s">
-        <v>235</v>
-      </c>
-      <c r="T8" t="s">
-        <v>133</v>
-      </c>
-      <c r="U8" t="s">
-        <v>244</v>
-      </c>
-      <c r="V8" t="s">
-        <v>144</v>
-      </c>
-      <c r="W8" t="s">
-        <v>249</v>
-      </c>
-      <c r="X8" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>254</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>164</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>260</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>175</v>
-      </c>
-      <c r="AC8" t="s">
-        <v>271</v>
+        <v>59</v>
+      </c>
+      <c r="R8">
+        <v>364</v>
+      </c>
+      <c r="S8">
+        <v>9</v>
+      </c>
+      <c r="T8">
+        <v>10.51</v>
+      </c>
+      <c r="U8">
+        <v>0.2</v>
+      </c>
+      <c r="V8">
+        <v>67</v>
+      </c>
+      <c r="W8">
+        <v>5</v>
+      </c>
+      <c r="X8">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="Y8">
+        <v>0.18</v>
+      </c>
+      <c r="Z8">
+        <v>1063</v>
+      </c>
+      <c r="AA8">
+        <v>150</v>
+      </c>
+      <c r="AB8">
+        <v>1987</v>
+      </c>
+      <c r="AC8">
+        <v>55</v>
       </c>
       <c r="AD8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AH8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AI8" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:35">
       <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" t="s">
-        <v>196</v>
-      </c>
-      <c r="D9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E9" t="s">
-        <v>200</v>
+      <c r="B9">
+        <v>0.01</v>
+      </c>
+      <c r="C9">
+        <v>0.00019</v>
+      </c>
+      <c r="D9">
+        <v>0.005</v>
+      </c>
+      <c r="E9">
+        <v>0.0022</v>
       </c>
       <c r="F9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G9" t="s">
-        <v>75</v>
-      </c>
-      <c r="H9" t="s">
-        <v>81</v>
-      </c>
-      <c r="I9" t="s">
-        <v>210</v>
-      </c>
-      <c r="J9" t="s">
-        <v>92</v>
-      </c>
-      <c r="K9" t="s">
-        <v>219</v>
-      </c>
-      <c r="L9" t="s">
-        <v>103</v>
-      </c>
-      <c r="M9" t="s">
-        <v>212</v>
-      </c>
-      <c r="N9" t="s">
-        <v>111</v>
-      </c>
-      <c r="O9" t="s">
-        <v>231</v>
+        <v>59</v>
+      </c>
+      <c r="H9">
+        <v>3.31</v>
+      </c>
+      <c r="I9">
+        <v>0.05</v>
+      </c>
+      <c r="J9">
+        <v>4768</v>
+      </c>
+      <c r="K9">
+        <v>57</v>
+      </c>
+      <c r="L9">
+        <v>0.5</v>
+      </c>
+      <c r="M9">
+        <v>0.08</v>
+      </c>
+      <c r="N9">
+        <v>2.9</v>
+      </c>
+      <c r="O9">
+        <v>0.9</v>
       </c>
       <c r="P9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q9" t="s">
-        <v>75</v>
-      </c>
-      <c r="R9" t="s">
-        <v>123</v>
-      </c>
-      <c r="S9" t="s">
-        <v>188</v>
-      </c>
-      <c r="T9" t="s">
-        <v>134</v>
-      </c>
-      <c r="U9" t="s">
-        <v>102</v>
-      </c>
-      <c r="V9" t="s">
-        <v>145</v>
-      </c>
-      <c r="W9" t="s">
-        <v>250</v>
-      </c>
-      <c r="X9" t="s">
-        <v>155</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>255</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>165</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>261</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>176</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>144</v>
+        <v>59</v>
+      </c>
+      <c r="R9">
+        <v>1522</v>
+      </c>
+      <c r="S9">
+        <v>32</v>
+      </c>
+      <c r="T9">
+        <v>14.83</v>
+      </c>
+      <c r="U9">
+        <v>0.28</v>
+      </c>
+      <c r="V9">
+        <v>95</v>
+      </c>
+      <c r="W9">
+        <v>7</v>
+      </c>
+      <c r="X9">
+        <v>0.9</v>
+      </c>
+      <c r="Y9">
+        <v>0.23</v>
+      </c>
+      <c r="Z9">
+        <v>1491</v>
+      </c>
+      <c r="AA9">
+        <v>203</v>
+      </c>
+      <c r="AB9">
+        <v>2262</v>
+      </c>
+      <c r="AC9">
+        <v>67</v>
       </c>
       <c r="AD9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF9" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG9" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>249</v>
+        <v>59</v>
+      </c>
+      <c r="AH9">
+        <v>16</v>
+      </c>
+      <c r="AI9">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" t="s">
-        <v>192</v>
-      </c>
-      <c r="D10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" t="s">
-        <v>199</v>
+      <c r="B10">
+        <v>0.013</v>
+      </c>
+      <c r="C10">
+        <v>0.00025</v>
+      </c>
+      <c r="D10">
+        <v>0.008</v>
+      </c>
+      <c r="E10">
+        <v>0.0025</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" t="s">
-        <v>82</v>
-      </c>
-      <c r="I10" t="s">
-        <v>212</v>
-      </c>
-      <c r="J10" t="s">
-        <v>93</v>
-      </c>
-      <c r="K10" t="s">
-        <v>220</v>
-      </c>
-      <c r="L10" t="s">
-        <v>104</v>
-      </c>
-      <c r="M10" t="s">
-        <v>224</v>
-      </c>
-      <c r="N10" t="s">
-        <v>114</v>
-      </c>
-      <c r="O10" t="s">
-        <v>230</v>
+        <v>59</v>
+      </c>
+      <c r="H10">
+        <v>5.63</v>
+      </c>
+      <c r="I10">
+        <v>0.08</v>
+      </c>
+      <c r="J10">
+        <v>8733</v>
+      </c>
+      <c r="K10">
+        <v>94</v>
+      </c>
+      <c r="L10">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="M10">
+        <v>0.1</v>
+      </c>
+      <c r="N10">
+        <v>5</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
       </c>
       <c r="P10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q10" t="s">
-        <v>75</v>
-      </c>
-      <c r="R10" t="s">
-        <v>124</v>
-      </c>
-      <c r="S10" t="s">
-        <v>217</v>
-      </c>
-      <c r="T10" t="s">
-        <v>135</v>
-      </c>
-      <c r="U10" t="s">
-        <v>242</v>
-      </c>
-      <c r="V10" t="s">
-        <v>146</v>
-      </c>
-      <c r="W10" t="s">
-        <v>234</v>
-      </c>
-      <c r="X10" t="s">
-        <v>156</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>252</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>262</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>272</v>
+        <v>59</v>
+      </c>
+      <c r="R10">
+        <v>2214</v>
+      </c>
+      <c r="S10">
+        <v>46</v>
+      </c>
+      <c r="T10">
+        <v>18.6</v>
+      </c>
+      <c r="U10">
+        <v>0.3</v>
+      </c>
+      <c r="V10">
+        <v>275</v>
+      </c>
+      <c r="W10">
+        <v>14</v>
+      </c>
+      <c r="X10">
+        <v>1.25</v>
+      </c>
+      <c r="Y10">
+        <v>0.29</v>
+      </c>
+      <c r="Z10">
+        <v>2071</v>
+      </c>
+      <c r="AA10">
+        <v>274</v>
+      </c>
+      <c r="AB10">
+        <v>2764</v>
+      </c>
+      <c r="AC10">
+        <v>84</v>
       </c>
       <c r="AD10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG10" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH10" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="AH10">
+        <v>21</v>
+      </c>
+      <c r="AI10">
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:35">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" t="s">
-        <v>193</v>
-      </c>
-      <c r="D11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" t="s">
-        <v>203</v>
+      <c r="B11">
+        <v>0.012</v>
+      </c>
+      <c r="C11">
+        <v>0.00023</v>
+      </c>
+      <c r="D11">
+        <v>0.012</v>
+      </c>
+      <c r="E11">
+        <v>0.003</v>
       </c>
       <c r="F11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G11" t="s">
-        <v>75</v>
-      </c>
-      <c r="H11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11">
+        <v>3.88</v>
+      </c>
+      <c r="I11">
+        <v>0.06</v>
+      </c>
+      <c r="J11">
+        <v>7525</v>
+      </c>
+      <c r="K11">
         <v>83</v>
       </c>
-      <c r="I11" t="s">
-        <v>213</v>
-      </c>
-      <c r="J11" t="s">
-        <v>94</v>
-      </c>
-      <c r="K11" t="s">
-        <v>216</v>
-      </c>
-      <c r="L11" t="s">
-        <v>105</v>
-      </c>
-      <c r="M11" t="s">
-        <v>227</v>
-      </c>
-      <c r="N11" t="s">
-        <v>115</v>
-      </c>
-      <c r="O11" t="s">
-        <v>232</v>
+      <c r="L11">
+        <v>1.21</v>
+      </c>
+      <c r="M11">
+        <v>0.16</v>
+      </c>
+      <c r="N11">
+        <v>16</v>
+      </c>
+      <c r="O11">
+        <v>4</v>
       </c>
       <c r="P11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q11" t="s">
-        <v>75</v>
-      </c>
-      <c r="R11" t="s">
-        <v>125</v>
-      </c>
-      <c r="S11" t="s">
-        <v>236</v>
-      </c>
-      <c r="T11" t="s">
-        <v>136</v>
-      </c>
-      <c r="U11" t="s">
-        <v>245</v>
-      </c>
-      <c r="V11" t="s">
-        <v>147</v>
-      </c>
-      <c r="W11" t="s">
-        <v>185</v>
-      </c>
-      <c r="X11" t="s">
-        <v>157</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>245</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>167</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>263</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>178</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>273</v>
+        <v>59</v>
+      </c>
+      <c r="R11">
+        <v>4323</v>
+      </c>
+      <c r="S11">
+        <v>89</v>
+      </c>
+      <c r="T11">
+        <v>19</v>
+      </c>
+      <c r="U11">
+        <v>0.4</v>
+      </c>
+      <c r="V11">
+        <v>179</v>
+      </c>
+      <c r="W11">
+        <v>10</v>
+      </c>
+      <c r="X11">
+        <v>1.8</v>
+      </c>
+      <c r="Y11">
+        <v>0.4</v>
+      </c>
+      <c r="Z11">
+        <v>2080</v>
+      </c>
+      <c r="AA11">
+        <v>271</v>
+      </c>
+      <c r="AB11">
+        <v>2530</v>
+      </c>
+      <c r="AC11">
+        <v>78</v>
       </c>
       <c r="AD11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF11" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG11" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH11" t="s">
-        <v>187</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>250</v>
+        <v>59</v>
+      </c>
+      <c r="AH11">
+        <v>25</v>
+      </c>
+      <c r="AI11">
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:35">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" t="s">
-        <v>197</v>
-      </c>
-      <c r="D12" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" t="s">
-        <v>204</v>
+      <c r="B12">
+        <v>0.014</v>
+      </c>
+      <c r="C12">
+        <v>0.00027</v>
+      </c>
+      <c r="D12">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E12">
+        <v>0.0029</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G12" t="s">
-        <v>75</v>
-      </c>
-      <c r="H12" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12" t="s">
-        <v>212</v>
-      </c>
-      <c r="J12" t="s">
-        <v>95</v>
-      </c>
-      <c r="K12" t="s">
-        <v>221</v>
-      </c>
-      <c r="L12" t="s">
-        <v>106</v>
-      </c>
-      <c r="M12" t="s">
-        <v>228</v>
-      </c>
-      <c r="N12" t="s">
-        <v>116</v>
-      </c>
-      <c r="O12" t="s">
-        <v>109</v>
+        <v>59</v>
+      </c>
+      <c r="H12">
+        <v>5.71</v>
+      </c>
+      <c r="I12">
+        <v>0.08</v>
+      </c>
+      <c r="J12">
+        <v>10334</v>
+      </c>
+      <c r="K12">
+        <v>110</v>
+      </c>
+      <c r="L12">
+        <v>0.99</v>
+      </c>
+      <c r="M12">
+        <v>0.14</v>
+      </c>
+      <c r="N12">
+        <v>9</v>
+      </c>
+      <c r="O12">
+        <v>2</v>
       </c>
       <c r="P12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q12" t="s">
-        <v>75</v>
-      </c>
-      <c r="R12" t="s">
-        <v>126</v>
-      </c>
-      <c r="S12" t="s">
+        <v>59</v>
+      </c>
+      <c r="R12">
+        <v>4519</v>
+      </c>
+      <c r="S12">
+        <v>93</v>
+      </c>
+      <c r="T12">
+        <v>24.8</v>
+      </c>
+      <c r="U12">
+        <v>0.5</v>
+      </c>
+      <c r="V12">
         <v>237</v>
       </c>
-      <c r="T12" t="s">
-        <v>137</v>
-      </c>
-      <c r="U12" t="s">
-        <v>240</v>
-      </c>
-      <c r="V12" t="s">
-        <v>148</v>
-      </c>
-      <c r="W12" t="s">
-        <v>251</v>
-      </c>
-      <c r="X12" t="s">
-        <v>158</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>168</v>
-      </c>
-      <c r="AA12" t="s">
-        <v>264</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>179</v>
-      </c>
-      <c r="AC12" t="s">
-        <v>236</v>
+      <c r="W12">
+        <v>12</v>
+      </c>
+      <c r="X12">
+        <v>1.5</v>
+      </c>
+      <c r="Y12">
+        <v>0.3</v>
+      </c>
+      <c r="Z12">
+        <v>2417</v>
+      </c>
+      <c r="AA12">
+        <v>316</v>
+      </c>
+      <c r="AB12">
+        <v>2707</v>
+      </c>
+      <c r="AC12">
+        <v>89</v>
       </c>
       <c r="AD12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF12" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG12" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH12" t="s">
-        <v>188</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>247</v>
+        <v>59</v>
+      </c>
+      <c r="AH12">
+        <v>32</v>
+      </c>
+      <c r="AI12">
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:35">
       <c r="A13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" t="s">
-        <v>197</v>
-      </c>
-      <c r="D13" t="s">
-        <v>72</v>
-      </c>
-      <c r="E13" t="s">
-        <v>205</v>
+      <c r="B13">
+        <v>0.014</v>
+      </c>
+      <c r="C13">
+        <v>0.00027</v>
+      </c>
+      <c r="D13">
+        <v>0.01</v>
+      </c>
+      <c r="E13">
+        <v>0.0027</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>85</v>
-      </c>
-      <c r="I13" t="s">
-        <v>209</v>
-      </c>
-      <c r="J13" t="s">
-        <v>96</v>
-      </c>
-      <c r="K13" t="s">
-        <v>222</v>
-      </c>
-      <c r="L13" t="s">
-        <v>107</v>
-      </c>
-      <c r="M13" t="s">
-        <v>224</v>
-      </c>
-      <c r="N13" t="s">
-        <v>110</v>
-      </c>
-      <c r="O13" t="s">
-        <v>230</v>
+        <v>59</v>
+      </c>
+      <c r="H13">
+        <v>5.04</v>
+      </c>
+      <c r="I13">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J13">
+        <v>10570</v>
+      </c>
+      <c r="K13">
+        <v>112</v>
+      </c>
+      <c r="L13">
+        <v>0.62</v>
+      </c>
+      <c r="M13">
+        <v>0.1</v>
+      </c>
+      <c r="N13">
+        <v>3</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
       </c>
       <c r="P13" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q13" t="s">
-        <v>75</v>
-      </c>
-      <c r="R13" t="s">
-        <v>127</v>
-      </c>
-      <c r="S13" t="s">
-        <v>238</v>
-      </c>
-      <c r="T13" t="s">
-        <v>138</v>
-      </c>
-      <c r="U13" t="s">
-        <v>240</v>
-      </c>
-      <c r="V13" t="s">
-        <v>149</v>
-      </c>
-      <c r="W13" t="s">
-        <v>185</v>
-      </c>
-      <c r="X13" t="s">
-        <v>159</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>169</v>
-      </c>
-      <c r="AA13" t="s">
-        <v>265</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>180</v>
-      </c>
-      <c r="AC13" t="s">
-        <v>274</v>
+        <v>59</v>
+      </c>
+      <c r="R13">
+        <v>1608</v>
+      </c>
+      <c r="S13">
+        <v>34</v>
+      </c>
+      <c r="T13">
+        <v>24.1</v>
+      </c>
+      <c r="U13">
+        <v>0.5</v>
+      </c>
+      <c r="V13">
+        <v>172</v>
+      </c>
+      <c r="W13">
+        <v>10</v>
+      </c>
+      <c r="X13">
+        <v>1.3</v>
+      </c>
+      <c r="Y13">
+        <v>0.3</v>
+      </c>
+      <c r="Z13">
+        <v>2385</v>
+      </c>
+      <c r="AA13">
+        <v>309</v>
+      </c>
+      <c r="AB13">
+        <v>2773</v>
+      </c>
+      <c r="AC13">
+        <v>88</v>
       </c>
       <c r="AD13" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE13" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF13" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG13" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH13" t="s">
-        <v>189</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="AH13">
+        <v>18</v>
+      </c>
+      <c r="AI13">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:35">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" t="s">
-        <v>192</v>
-      </c>
-      <c r="D14" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" t="s">
-        <v>206</v>
+      <c r="B14">
+        <v>0.013</v>
+      </c>
+      <c r="C14">
+        <v>0.00025</v>
+      </c>
+      <c r="D14">
+        <v>0.007</v>
+      </c>
+      <c r="E14">
+        <v>0.0023</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H14" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" t="s">
-        <v>213</v>
-      </c>
-      <c r="J14" t="s">
-        <v>97</v>
-      </c>
-      <c r="K14" t="s">
-        <v>223</v>
-      </c>
-      <c r="L14" t="s">
-        <v>108</v>
-      </c>
-      <c r="M14" t="s">
-        <v>224</v>
-      </c>
-      <c r="N14" t="s">
-        <v>117</v>
-      </c>
-      <c r="O14" t="s">
-        <v>231</v>
+        <v>59</v>
+      </c>
+      <c r="H14">
+        <v>3.64</v>
+      </c>
+      <c r="I14">
+        <v>0.06</v>
+      </c>
+      <c r="J14">
+        <v>8363</v>
+      </c>
+      <c r="K14">
+        <v>91</v>
+      </c>
+      <c r="L14">
+        <v>0.6</v>
+      </c>
+      <c r="M14">
+        <v>0.1</v>
+      </c>
+      <c r="N14">
+        <v>2.6</v>
+      </c>
+      <c r="O14">
+        <v>0.9</v>
       </c>
       <c r="P14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="Q14" t="s">
-        <v>75</v>
-      </c>
-      <c r="R14" t="s">
-        <v>128</v>
-      </c>
-      <c r="S14" t="s">
-        <v>239</v>
-      </c>
-      <c r="T14" t="s">
-        <v>139</v>
-      </c>
-      <c r="U14" t="s">
-        <v>245</v>
-      </c>
-      <c r="V14" t="s">
-        <v>150</v>
-      </c>
-      <c r="W14" t="s">
-        <v>247</v>
-      </c>
-      <c r="X14" t="s">
-        <v>158</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>242</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>170</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>266</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>181</v>
-      </c>
-      <c r="AC14" t="s">
-        <v>275</v>
+        <v>59</v>
+      </c>
+      <c r="R14">
+        <v>1344</v>
+      </c>
+      <c r="S14">
+        <v>29</v>
+      </c>
+      <c r="T14">
+        <v>21.9</v>
+      </c>
+      <c r="U14">
+        <v>0.4</v>
+      </c>
+      <c r="V14">
+        <v>131</v>
+      </c>
+      <c r="W14">
+        <v>8</v>
+      </c>
+      <c r="X14">
+        <v>1.5</v>
+      </c>
+      <c r="Y14">
+        <v>0.3</v>
+      </c>
+      <c r="Z14">
+        <v>1831</v>
+      </c>
+      <c r="AA14">
+        <v>248</v>
+      </c>
+      <c r="AB14">
+        <v>2272</v>
+      </c>
+      <c r="AC14">
+        <v>76</v>
       </c>
       <c r="AD14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AE14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AF14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="AG14" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH14" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI14" t="s">
-        <v>250</v>
+        <v>59</v>
+      </c>
+      <c r="AH14">
+        <v>23</v>
+      </c>
+      <c r="AI14">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>